<commit_message>
feat: update predictive analytics model with Weibull hazard scoring, Ising coupling, and regime detection
</commit_message>
<xml_diff>
--- a/baloto.xlsx
+++ b/baloto.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1022"/>
+  <dimension ref="A1:J1023"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35181,6 +35181,40 @@
       </c>
       <c r="J1022" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="n">
+        <v>2717</v>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="C1023" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1023" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1023" t="n">
+        <v>14</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1023" t="n">
+        <v>31</v>
+      </c>
+      <c r="H1023" t="n">
+        <v>10</v>
+      </c>
+      <c r="I1023" t="n">
+        <v>61600000000</v>
+      </c>
+      <c r="J1023" t="n">
+        <v>67008550</v>
       </c>
     </row>
   </sheetData>
@@ -35194,7 +35228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1009"/>
+  <dimension ref="A1:J1010"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69521,6 +69555,40 @@
         <v>22054450</v>
       </c>
     </row>
+    <row r="1010">
+      <c r="A1010" t="n">
+        <v>2717</v>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="C1010" t="n">
+        <v>19</v>
+      </c>
+      <c r="D1010" t="n">
+        <v>23</v>
+      </c>
+      <c r="E1010" t="n">
+        <v>27</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>38</v>
+      </c>
+      <c r="G1010" t="n">
+        <v>40</v>
+      </c>
+      <c r="H1010" t="n">
+        <v>14</v>
+      </c>
+      <c r="I1010" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1010" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>